<commit_message>
new start from v10
</commit_message>
<xml_diff>
--- a/Data/exogenous_data/Finland_MASTER_Calibration_old_UPDATED.xlsx
+++ b/Data/exogenous_data/Finland_MASTER_Calibration_old_UPDATED.xlsx
@@ -6468,7 +6468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="12" customWidth="1" style="11" min="1" max="1"/>
@@ -6878,6 +6878,33 @@
       <c r="E15" t="inlineStr">
         <is>
           <t>Priority-ranked calibration fixes based on model vs reality gaps</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Copilot</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Nuclear thermal efficiency corrected: URANIUM ratio -2.7027 → -3.125 (37% → 32%)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Data/2017/00_INDEP/Layers_in_out.csv (NUCLEAR + NUCLEAR_SMR rows)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Finnish plants (Loviisa PWR + Olkiluoto BWR, 1970s-80s vintage) operate at ~32%. Fixes PE_nuclear underestimation (56 → ~65 TWh). Also applied to NUCLEAR_SMR for consistency.</t>
         </is>
       </c>
     </row>
@@ -11936,6 +11963,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -11980,7 +12008,7 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>-2.7027</v>
+        <v>-3.125</v>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
@@ -11988,7 +12016,7 @@
         </is>
       </c>
       <c r="E4" s="4" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="F4" s="4" t="n"/>
     </row>

</xml_diff>